<commit_message>
feat(linkedin-scraper): 186 keywords (las 4 de Upwork) con rotación 15/corrida
Carga el set completo de keywords de los 4 scrapers de Upwork (Market/Automation-BI/
Business/Financial, deduplicado = 186) en el scraper de LinkedIn, con rotación por
$getWorkflowStaticData (15 por corrida, ciclo ~2 días) para no gatillar el 429 del
guest API. Filtro 1099-US y fit del classifier SIN cambios. Excel de criterios+keywords
actualizado con las 186.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/linkedin jobs/LinkedIn - Criterios y Keywords.xlsx
+++ b/linkedin jobs/LinkedIn - Criterios y Keywords.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criterios" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords por BU" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Solapas y Estados" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -46,7 +46,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -56,6 +56,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F1E1B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ECECE8"/>
       </patternFill>
     </fill>
   </fills>
@@ -85,12 +90,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -98,6 +101,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -463,13 +469,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="64" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -519,7 +525,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Filtro duro en búsqueda + en el parseo por location/estado</t>
+          <t>Filtro duro (location/estado). No se saca nunca.</t>
         </is>
       </c>
     </row>
@@ -541,7 +547,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>La búsqueda ya restringe a contract; por eso las keywords van 'base'</t>
+          <t>La búsqueda ya restringe a contract → keywords van 'base'.</t>
         </is>
       </c>
     </row>
@@ -563,7 +569,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>'1099' en LinkedIn = contract sin W2 (la palabra casi nunca aparece literal)</t>
+          <t>'1099' en LinkedIn = contract sin W2.</t>
         </is>
       </c>
     </row>
@@ -585,139 +591,157 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Se puede achicar a 24h si se quiere más fresco</t>
+          <t>Se puede achicar a 24h.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Páginas por keyword</t>
+          <t>Keywords de búsqueda</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>186 (mismas que los 4 scrapers de Upwork)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Ajustable</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>1 página para cuidar el rate-limit (429) con muchas keywords</t>
+          <t>Ver hoja 'Keywords'.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Frecuencia del scraper</t>
+          <t>Rotación</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Cada 4 horas</t>
+          <t>15 keywords por corrida, rotando</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Ajustable</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Schedule trigger</t>
+          <t>LinkedIn (guest API) corta con 429; Upwork usa API oficial + tope 90. Ciclo completo ~13 corridas (~2 días).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Filtro de FIT</t>
+          <t>Páginas por keyword</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Classifier vs 8 Business Units (Claude Haiku)</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>FIJO</t>
+          <t>Ajustable</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Solo los FIT van a Check Proposal; el resto a Descartados</t>
+          <t>Cuida el rate-limit (429).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Rango de precio (salario)</t>
+          <t>Frecuencia del scraper</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Se captura cuando el job lo tiene</t>
+          <t>Cada 4 horas</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Columna 'Rango $'. ~13 de cada 21 lo traen; el resto queda vacío</t>
-        </is>
-      </c>
+          <t>Ajustable</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Auto-expirar viejos</t>
+          <t>Filtro de FIT</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Jobs &gt; 7 días → Descartados</t>
+          <t>Classifier vs 8 Business Units (Haiku)</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>FIJO</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>pg_cron 07:00 diario (migración 0035)</t>
+          <t>Solo FIT → Check Proposal; resto → Descartados.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Frecuencia classifier</t>
+          <t>Rango de precio</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Cada 4 horas (:15)</t>
+          <t>Se captura cuando el job lo tiene</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Ajustable</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Escalonado del de Upwork (:3/7/11...)</t>
+          <t>Columna 'Rango $' (compensation__salary). ~13/21 lo traen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Auto-expirar viejos</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Jobs &gt; 7 días → Descartados</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>pg_cron 07:00 (migración 0035).</t>
         </is>
       </c>
     </row>
@@ -732,144 +756,2273 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:C190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Keywords de búsqueda (nodo Config → searches)</t>
+          <t>Keywords de búsqueda del scraper de LinkedIn (= las 4 de Upwork)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>25 búsquedas · 1 página c/u · todas pasan igual por el filtro 1099-US + fit</t>
+          <t>186 keywords · 1 página c/u · rotan 15 por corrida · todas pasan igual por 1099-US + fit</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>total: 186</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Business Unit</t>
+          <t>Grupo (scraper Upwork)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Keywords</t>
+          <t>Keyword</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Genéricas (catch-all)</t>
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Genéricas</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>1099 contractor · independent contractor</t>
+          <t>1099 contractor</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Finance &amp; Accounting</t>
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Genéricas</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>fractional CFO · FP&amp;A · financial modeling · financial modeling contract · financial analyst</t>
+          <t>independent contractor</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Project Management &amp; BI</t>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>data analyst · data analyst contract · Power BI · Tableau · Looker Studio · Looker Studio contract</t>
+          <t>CFO</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>AI &amp; Automation</t>
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>AI consultant · machine learning engineer</t>
+          <t>Financial Analyst</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>System Integrations</t>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>n8n · Zapier · integration consultant</t>
+          <t>Head of Finance</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Sales &amp; Customer Success</t>
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>HubSpot consultant · lead generation</t>
+          <t>Finance Director</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Marketing &amp; Brand</t>
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Meta ads · SEO consultant</t>
+          <t>Financial Consultant</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Digital Experience &amp; Product</t>
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Webflow developer · Shopify developer</t>
+          <t>Financial Advisor</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Business Operations &amp; Back-Office</t>
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>ERP consultant</t>
+          <t>Financial Controller</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Financial Modeler</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Financial Models</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Forecast</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Cashflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Profit and Loss</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Financial Statement</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Profitability</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Balance Sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Valuation</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Mergers and Acquisitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>IRR</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>MOIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>DCF</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Business Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Business Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Pitch Deck</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Business Model</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>One pager</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Financial Modelling</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Financial Projection</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Financial Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Financial Planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Financial Forecasting</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Financial Planning and Budgeting</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Financial Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Fathom HQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Floatapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Baremetrics</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Churnkey</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Triple Whale</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Income Statement</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Scenario Planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Sensitivity Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Working Capital</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>Financial (finanzas)</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Inventory Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Warehouse Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Demand Planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Procurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>Vendor Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>Supply Chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Xfin</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Odoo</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Xero</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>QuickBooks</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>Netsuite</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>ServiceTitan</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>Service Titan</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>QBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>Bank Reconciliation</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Treasury Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>Corporate Advisory</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Invoice Automation</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>Bookkeeper</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>Chart of Accounts</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Books to Bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>Project Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>Notion</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>Clickup</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Asana</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Jira</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Business Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Business Development</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Business Operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Business Consulting</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>Pumping</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>Gyms</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>Laboratory</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="inlineStr">
+        <is>
+          <t>Business (ops/back-office/industrias)</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>Clinic</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>Reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>Business Intelligence</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>KPIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>Automation</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t>Scraping</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>LLM</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>C++</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>NLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>Algorithms</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>Git</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>AI Agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>LangChain</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>LangGraph</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>AutoGen</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
+        <is>
+          <t>Prompt Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B112" s="4" t="inlineStr">
+        <is>
+          <t>MCP</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B113" s="4" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B114" s="4" t="inlineStr">
+        <is>
+          <t>Power BI</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
+          <t>Looker Studio</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B116" s="4" t="inlineStr">
+        <is>
+          <t>Google Sheets</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B117" s="4" t="inlineStr">
+        <is>
+          <t>Make.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t>Low Code</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t>No Code</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B120" s="4" t="inlineStr">
+        <is>
+          <t>Airtable</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B121" s="4" t="inlineStr">
+        <is>
+          <t>Softr</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>N8N</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>Zapier</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>Power Automate</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B125" s="4" t="inlineStr">
+        <is>
+          <t>Big Query</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B126" s="4" t="inlineStr">
+        <is>
+          <t>Mysql</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B127" s="4" t="inlineStr">
+        <is>
+          <t>SQL</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B128" s="4" t="inlineStr">
+        <is>
+          <t>Pinecone</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B129" s="4" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B130" s="4" t="inlineStr">
+        <is>
+          <t>Snowflake</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B131" s="4" t="inlineStr">
+        <is>
+          <t>Data analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="6" t="inlineStr">
+        <is>
+          <t>Automation &amp; BI</t>
+        </is>
+      </c>
+      <c r="B132" s="4" t="inlineStr">
+        <is>
+          <t>Data Analytics</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B133" s="4" t="inlineStr">
+        <is>
+          <t>Web Development</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B134" s="4" t="inlineStr">
+        <is>
+          <t>Figma</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B135" s="4" t="inlineStr">
+        <is>
+          <t>Framer</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B136" s="4" t="inlineStr">
+        <is>
+          <t>Webflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B137" s="4" t="inlineStr">
+        <is>
+          <t>Wordpress</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B138" s="4" t="inlineStr">
+        <is>
+          <t>Woocommerce</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t>E-commerce development</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B140" s="4" t="inlineStr">
+        <is>
+          <t>Shopify</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B141" s="4" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B142" s="4" t="inlineStr">
+        <is>
+          <t>Hubspot</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B143" s="4" t="inlineStr">
+        <is>
+          <t>Zoho</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B144" s="4" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B145" s="4" t="inlineStr">
+        <is>
+          <t>Instantly</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B146" s="4" t="inlineStr">
+        <is>
+          <t>Manyreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B147" s="4" t="inlineStr">
+        <is>
+          <t>Manychat</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B148" s="4" t="inlineStr">
+        <is>
+          <t>Apollo</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B149" s="4" t="inlineStr">
+        <is>
+          <t>Email marketing</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B150" s="4" t="inlineStr">
+        <is>
+          <t>Lead Gen</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B151" s="4" t="inlineStr">
+        <is>
+          <t>Kommo</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B152" s="4" t="inlineStr">
+        <is>
+          <t>Bounceban</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B153" s="4" t="inlineStr">
+        <is>
+          <t>Twilio</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B154" s="4" t="inlineStr">
+        <is>
+          <t>Maildoso</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B155" s="4" t="inlineStr">
+        <is>
+          <t>Klaviyo</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B156" s="4" t="inlineStr">
+        <is>
+          <t>Gohighlevel</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t>Lemlist</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B158" s="4" t="inlineStr">
+        <is>
+          <t>Clay</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B159" s="4" t="inlineStr">
+        <is>
+          <t>Cursor</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B160" s="4" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B161" s="4" t="inlineStr">
+        <is>
+          <t>Lovable</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B162" s="4" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B163" s="4" t="inlineStr">
+        <is>
+          <t>App development</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B164" s="4" t="inlineStr">
+        <is>
+          <t>Bolt</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B165" s="4" t="inlineStr">
+        <is>
+          <t>Metricool</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B166" s="4" t="inlineStr">
+        <is>
+          <t>Supermetrics</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B167" s="4" t="inlineStr">
+        <is>
+          <t>Gamma</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B168" s="4" t="inlineStr">
+        <is>
+          <t>Canva</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B169" s="4" t="inlineStr">
+        <is>
+          <t>Liveplan</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B170" s="4" t="inlineStr">
+        <is>
+          <t>Campaign Outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B171" s="4" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B172" s="4" t="inlineStr">
+        <is>
+          <t>Linkedin Ads</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B173" s="4" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B174" s="4" t="inlineStr">
+        <is>
+          <t>Tiktok Ads</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B175" s="4" t="inlineStr">
+        <is>
+          <t>Hootsuite</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B176" s="4" t="inlineStr">
+        <is>
+          <t>Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B177" s="4" t="inlineStr">
+        <is>
+          <t>Social Media Analytics</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B178" s="4" t="inlineStr">
+        <is>
+          <t>Social Media Reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B179" s="4" t="inlineStr">
+        <is>
+          <t>Social Media Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B180" s="4" t="inlineStr">
+        <is>
+          <t>Content Calendar</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B181" s="4" t="inlineStr">
+        <is>
+          <t>Social Media Automation</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B182" s="4" t="inlineStr">
+        <is>
+          <t>Google Analytics GA4</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B183" s="4" t="inlineStr">
+        <is>
+          <t>Go-to-Market Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B184" s="4" t="inlineStr">
+        <is>
+          <t>GTM Framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B185" s="4" t="inlineStr">
+        <is>
+          <t>Market Entry Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B186" s="4" t="inlineStr">
+        <is>
+          <t>Product Launch Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B187" s="4" t="inlineStr">
+        <is>
+          <t>Growth Strategy Consultant</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B188" s="4" t="inlineStr">
+        <is>
+          <t>Commercial Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B189" s="4" t="inlineStr">
+        <is>
+          <t>Revenue Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="6" t="inlineStr">
+        <is>
+          <t>Market (web/marketing/sales/growth)</t>
+        </is>
+      </c>
+      <c r="B190" s="4" t="inlineStr">
+        <is>
+          <t>Pricing &amp; Packaging Strategy</t>
         </is>
       </c>
     </row>
@@ -889,13 +3042,13 @@
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Solapas de la UI y qué muestran</t>
+          <t>Solapas de la UI</t>
         </is>
       </c>
     </row>
@@ -929,7 +3082,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Solo los que hacen FIT con SWL. Tu lista de trabajo real</t>
+          <t>Solo los que hacen FIT con SWL. Tu lista de trabajo.</t>
         </is>
       </c>
     </row>
@@ -946,7 +3099,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Los que ya aplicaste en LinkedIn</t>
+          <t>Los que ya aplicaste en LinkedIn.</t>
         </is>
       </c>
     </row>
@@ -963,7 +3116,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Sin fit (classifier) + los que descartás a mano</t>
+          <t>Sin fit (classifier) + descartados a mano.</t>
         </is>
       </c>
     </row>
@@ -980,7 +3133,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Desglose por estado (Check Proposal / Sent / Sin fit / Descartados)</t>
+          <t>Desglose por estado.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
doc(linkedin): Excel sin header negro, título simple
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/linkedin jobs/LinkedIn - Criterios y Keywords.xlsx
+++ b/linkedin jobs/LinkedIn - Criterios y Keywords.xlsx
@@ -523,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -537,1233 +537,1209 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Referencia Colores:</t>
-        </is>
-      </c>
-      <c r="B1" s="7" t="inlineStr">
-        <is>
-          <t>Verde: en uso</t>
-        </is>
-      </c>
-      <c r="C1" s="7" t="inlineStr"/>
-      <c r="D1" s="7" t="inlineStr">
-        <is>
-          <t>1099 + US: SÍ o SÍ (fijo)</t>
-        </is>
-      </c>
-      <c r="E1" s="7" t="inlineStr"/>
-      <c r="F1" s="7" t="inlineStr"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr"/>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>Todas rotan 15 por corrida</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr"/>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>Ciclo completo ~2 días</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr"/>
-      <c r="F2" s="7" t="inlineStr"/>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>LinkedIn — Search Fields (keywords = mismas que Upwork)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Corporate Advisory (Finanzas):</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 1)</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 2)</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 3)</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 4)</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 5)</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 6)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>Corporate Advisory (Finanzas):</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 1)</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 2)</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 3)</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 4)</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 5)</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 6)</t>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Forecast</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Valuation</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Business Plan</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>Financial Modelling</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Fathom HQ</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>CFO</t>
+          <t>Financial Analyst</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Forecast</t>
+          <t>Cashflow</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Mergers and Acquisitions</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>Business Plan</t>
+          <t>Business Analysis</t>
         </is>
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>Financial Modelling</t>
+          <t>Financial Projection</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>Fathom HQ</t>
+          <t>Floatapp</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>Financial Analyst</t>
+          <t>Head of Finance</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Cashflow</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Mergers and Acquisitions</t>
+          <t>IRR</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>Business Analysis</t>
+          <t>Pitch Deck</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>Financial Projection</t>
+          <t>Financial Analysis</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>Floatapp</t>
+          <t>Baremetrics</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>Head of Finance</t>
+          <t>Finance Director</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>Profit and Loss</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>IRR</t>
+          <t>MOIC</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>Pitch Deck</t>
+          <t>Business Model</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>Financial Analysis</t>
+          <t>Financial Planning</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>Baremetrics</t>
+          <t>Churnkey</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>Finance Director</t>
+          <t>Financial Consultant</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>Profit and Loss</t>
+          <t>Financial Statement</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>MOIC</t>
+          <t>DCF</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
         <is>
-          <t>Business Model</t>
+          <t>One pager</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>Financial Planning</t>
+          <t>Financial Forecasting</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>Churnkey</t>
+          <t>Triple Whale</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Financial Consultant</t>
+          <t>Financial Advisor</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>Financial Statement</t>
+          <t>Profitability</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>DCF</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="inlineStr">
-        <is>
-          <t>One pager</t>
+          <t>EBITDA</t>
         </is>
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>Financial Forecasting</t>
+          <t>Financial Planning and Budgeting</t>
         </is>
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>Triple Whale</t>
+          <t>Income Statement</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Financial Advisor</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>Profitability</t>
+          <t>Balance Sheet</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>EBITDA</t>
+          <t>Net Income</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>Financial Planning and Budgeting</t>
+          <t>Financial Review</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>Income Statement</t>
+          <t>Scenario Planning</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Financial Controller</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>Balance Sheet</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>Net Income</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>Financial Review</t>
+          <t>Financial Modeler</t>
         </is>
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>Scenario Planning</t>
+          <t>Sensitivity Analysis</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Financial Modeler</t>
+          <t>Financial Models</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>Sensitivity Analysis</t>
+          <t>Working Capital</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Financial Models</t>
-        </is>
-      </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>Working Capital</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="G14" s="10" t="inlineStr">
-        <is>
           <t>Private Equity</t>
         </is>
       </c>
     </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Business Mastery (Ops / Back-office):</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 1)</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 2)</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 3)</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 4)</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 5)</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 6)</t>
+        </is>
+      </c>
+    </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>Business Mastery (Ops / Back-office):</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 1)</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 2)</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 3)</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 4)</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 5)</t>
-        </is>
-      </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 6)</t>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Inventory Management</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Xfin</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>Bank Reconciliation</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>Project Management</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Business Strategy</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Inventory Management</t>
+          <t>Warehouse Management</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>Xfin</t>
+          <t>Odoo</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>Bank Reconciliation</t>
+          <t>Treasury Management</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>Project Management</t>
+          <t>Notion</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>Business Strategy</t>
+          <t>Business Development</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Real Estate</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Warehouse Management</t>
+          <t>Demand Planning</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>Odoo</t>
+          <t>Xero</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>Treasury Management</t>
+          <t>Revenue Management</t>
         </is>
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
-          <t>Notion</t>
+          <t>Clickup</t>
         </is>
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>Business Development</t>
+          <t>Business Operations</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>HVAC</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Demand Planning</t>
+          <t>Procurement</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>Xero</t>
+          <t>QuickBooks</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>Revenue Management</t>
+          <t>Corporate Advisory</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>Clickup</t>
+          <t>Asana</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>Business Operations</t>
+          <t>Business Consulting</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Pumping</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Procurement</t>
+          <t>Vendor Management</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>QuickBooks</t>
+          <t>Netsuite</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>Corporate Advisory</t>
+          <t>Invoice Automation</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>Asana</t>
-        </is>
-      </c>
-      <c r="F20" s="10" t="inlineStr">
-        <is>
-          <t>Business Consulting</t>
+          <t>Jira</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>Pumping</t>
+          <t>Plumbing</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Vendor Management</t>
+          <t>Supply Chain</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Netsuite</t>
+          <t>ServiceTitan</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>Invoice Automation</t>
-        </is>
-      </c>
-      <c r="E21" s="10" t="inlineStr">
-        <is>
-          <t>Jira</t>
+          <t>Bookkeeper</t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Gyms</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>Supply Chain</t>
-        </is>
-      </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>ServiceTitan</t>
+          <t>Service Titan</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>Bookkeeper</t>
+          <t>Chart of Accounts</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
-          <t>Gyms</t>
+          <t>Environmental</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>Service Titan</t>
+          <t>QBO</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>Chart of Accounts</t>
+          <t>Books to Bank</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
         <is>
-          <t>Environmental</t>
+          <t>Laboratory</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="C24" s="10" t="inlineStr">
-        <is>
-          <t>QBO</t>
-        </is>
-      </c>
-      <c r="D24" s="10" t="inlineStr">
-        <is>
-          <t>Books to Bank</t>
-        </is>
-      </c>
       <c r="G24" s="10" t="inlineStr">
         <is>
-          <t>Laboratory</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="G25" s="10" t="inlineStr">
-        <is>
           <t>Clinic</t>
         </is>
       </c>
     </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>Automation &amp; Business Intelligence:</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 1)</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 2)</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 3)</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 4)</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 5)</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 6)</t>
+        </is>
+      </c>
+    </row>
     <row r="27">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t>Automation &amp; Business Intelligence:</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 1)</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 2)</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 3)</t>
-        </is>
-      </c>
-      <c r="E27" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 4)</t>
-        </is>
-      </c>
-      <c r="F27" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 5)</t>
-        </is>
-      </c>
-      <c r="G27" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 6)</t>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Automation</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>Low Code</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>N8N</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>Big Query</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Reporting</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Automation</t>
+          <t>Integration</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>Tableau</t>
+          <t>Power BI</t>
         </is>
       </c>
       <c r="E28" s="10" t="inlineStr">
         <is>
-          <t>Low Code</t>
+          <t>No Code</t>
         </is>
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>N8N</t>
+          <t>Zapier</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>Big Query</t>
+          <t>Mysql</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>Reporting</t>
+          <t>Business Intelligence</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>Scraping</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>Power BI</t>
+          <t>Looker Studio</t>
         </is>
       </c>
       <c r="E29" s="10" t="inlineStr">
         <is>
-          <t>No Code</t>
+          <t>Airtable</t>
         </is>
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>Zapier</t>
+          <t>Power Automate</t>
         </is>
       </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
-          <t>Mysql</t>
+          <t>SQL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Business Intelligence</t>
+          <t>KPIS</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>Scraping</t>
+          <t>LLM</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>Looker Studio</t>
+          <t>Google Sheets</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr">
         <is>
-          <t>Airtable</t>
-        </is>
-      </c>
-      <c r="F30" s="10" t="inlineStr">
-        <is>
-          <t>Power Automate</t>
+          <t>Softr</t>
         </is>
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>SQL</t>
+          <t>Pinecone</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>KPIS</t>
-        </is>
-      </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>LLM</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>Google Sheets</t>
-        </is>
-      </c>
-      <c r="E31" s="10" t="inlineStr">
-        <is>
-          <t>Softr</t>
+          <t>Make.com</t>
         </is>
       </c>
       <c r="G31" s="10" t="inlineStr">
         <is>
-          <t>Pinecone</t>
+          <t>Supabase</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="D32" s="10" t="inlineStr">
-        <is>
-          <t>Make.com</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="G32" s="10" t="inlineStr">
         <is>
-          <t>Supabase</t>
+          <t>Snowflake</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>C++</t>
         </is>
       </c>
       <c r="G33" s="10" t="inlineStr">
         <is>
-          <t>Snowflake</t>
+          <t>Data analyst</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>C++</t>
+          <t>NLP</t>
         </is>
       </c>
       <c r="G34" s="10" t="inlineStr">
         <is>
-          <t>Data analyst</t>
+          <t>Data Analytics</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>NLP</t>
-        </is>
-      </c>
-      <c r="G35" s="10" t="inlineStr">
-        <is>
-          <t>Data Analytics</t>
+          <t>Algorithms</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>Algorithms</t>
+          <t>Git</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>AI Agents</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>AI Agents</t>
+          <t>LangChain</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>LangChain</t>
+          <t>LangGraph</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>LangGraph</t>
+          <t>AutoGen</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>AutoGen</t>
+          <t>RAG</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>Prompt Engineering</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>Prompt Engineering</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="C44" s="10" t="inlineStr">
-        <is>
           <t>MCP</t>
         </is>
       </c>
     </row>
+    <row r="44"/>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>Market Aceleration (Web / Marketing / Sales):</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 1)</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 2)</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 3)</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 4)</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 5)</t>
+        </is>
+      </c>
+      <c r="G45" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 6)</t>
+        </is>
+      </c>
+      <c r="H45" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 7)</t>
+        </is>
+      </c>
+    </row>
     <row r="46">
-      <c r="A46" s="8" t="inlineStr">
-        <is>
-          <t>Market Aceleration (Web / Marketing / Sales):</t>
-        </is>
-      </c>
-      <c r="B46" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 1)</t>
-        </is>
-      </c>
-      <c r="C46" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 2)</t>
-        </is>
-      </c>
-      <c r="D46" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 3)</t>
-        </is>
-      </c>
-      <c r="E46" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 4)</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 5)</t>
-        </is>
-      </c>
-      <c r="G46" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 6)</t>
-        </is>
-      </c>
-      <c r="H46" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 7)</t>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>Web Development</t>
+        </is>
+      </c>
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="D46" s="10" t="inlineStr">
+        <is>
+          <t>Apollo</t>
+        </is>
+      </c>
+      <c r="E46" s="10" t="inlineStr">
+        <is>
+          <t>Cursor</t>
+        </is>
+      </c>
+      <c r="F46" s="10" t="inlineStr">
+        <is>
+          <t>Metricool</t>
+        </is>
+      </c>
+      <c r="G46" s="10" t="inlineStr">
+        <is>
+          <t>Campaign Outreach</t>
+        </is>
+      </c>
+      <c r="H46" s="10" t="inlineStr">
+        <is>
+          <t>Go-to-Market Strategy</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>Web Development</t>
+          <t>Figma</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>Salesforce</t>
+          <t>Hubspot</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>Apollo</t>
+          <t>Email marketing</t>
         </is>
       </c>
       <c r="E47" s="10" t="inlineStr">
         <is>
-          <t>Cursor</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
-          <t>Metricool</t>
+          <t>Supermetrics</t>
         </is>
       </c>
       <c r="G47" s="10" t="inlineStr">
         <is>
-          <t>Campaign Outreach</t>
+          <t>Google Ads</t>
         </is>
       </c>
       <c r="H47" s="10" t="inlineStr">
         <is>
-          <t>Go-to-Market Strategy</t>
+          <t>GTM Framework</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>Figma</t>
+          <t>Framer</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
         <is>
-          <t>Hubspot</t>
+          <t>Zoho</t>
         </is>
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t>Email marketing</t>
+          <t>Lead Gen</t>
         </is>
       </c>
       <c r="E48" s="10" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="F48" s="10" t="inlineStr">
         <is>
-          <t>Supermetrics</t>
+          <t>Gamma</t>
         </is>
       </c>
       <c r="G48" s="10" t="inlineStr">
         <is>
-          <t>Google Ads</t>
+          <t>Linkedin Ads</t>
         </is>
       </c>
       <c r="H48" s="10" t="inlineStr">
         <is>
-          <t>GTM Framework</t>
+          <t>Market Entry Strategy</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>Framer</t>
+          <t>Webflow</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>Zoho</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>Lead Gen</t>
+          <t>Kommo</t>
         </is>
       </c>
       <c r="E49" s="10" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>v0</t>
         </is>
       </c>
       <c r="F49" s="10" t="inlineStr">
         <is>
-          <t>Gamma</t>
+          <t>Canva</t>
         </is>
       </c>
       <c r="G49" s="10" t="inlineStr">
         <is>
-          <t>Linkedin Ads</t>
+          <t>Meta Ads</t>
         </is>
       </c>
       <c r="H49" s="10" t="inlineStr">
         <is>
-          <t>Market Entry Strategy</t>
+          <t>Product Launch Strategy</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>Webflow</t>
+          <t>Wordpress</t>
         </is>
       </c>
       <c r="C50" s="10" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Instantly</t>
         </is>
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t>Kommo</t>
+          <t>Bounceban</t>
         </is>
       </c>
       <c r="E50" s="10" t="inlineStr">
         <is>
-          <t>v0</t>
+          <t>App development</t>
         </is>
       </c>
       <c r="F50" s="10" t="inlineStr">
         <is>
-          <t>Canva</t>
+          <t>Liveplan</t>
         </is>
       </c>
       <c r="G50" s="10" t="inlineStr">
         <is>
-          <t>Meta Ads</t>
+          <t>Tiktok Ads</t>
         </is>
       </c>
       <c r="H50" s="10" t="inlineStr">
         <is>
-          <t>Product Launch Strategy</t>
+          <t>Growth Strategy Consultant</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>Wordpress</t>
+          <t>Woocommerce</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>Instantly</t>
+          <t>Manyreach</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>Bounceban</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="E51" s="10" t="inlineStr">
         <is>
-          <t>App development</t>
-        </is>
-      </c>
-      <c r="F51" s="10" t="inlineStr">
-        <is>
-          <t>Liveplan</t>
+          <t>Bolt</t>
         </is>
       </c>
       <c r="G51" s="10" t="inlineStr">
         <is>
-          <t>Tiktok Ads</t>
+          <t>Hootsuite</t>
         </is>
       </c>
       <c r="H51" s="10" t="inlineStr">
         <is>
-          <t>Growth Strategy Consultant</t>
+          <t>Commercial Strategy</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>Woocommerce</t>
+          <t>E-commerce development</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
         <is>
-          <t>Manyreach</t>
+          <t>Manychat</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>Twilio</t>
-        </is>
-      </c>
-      <c r="E52" s="10" t="inlineStr">
-        <is>
-          <t>Bolt</t>
+          <t>Maildoso</t>
         </is>
       </c>
       <c r="G52" s="10" t="inlineStr">
         <is>
-          <t>Hootsuite</t>
+          <t>Buffer</t>
         </is>
       </c>
       <c r="H52" s="10" t="inlineStr">
         <is>
-          <t>Commercial Strategy</t>
+          <t>Revenue Strategy</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>E-commerce development</t>
-        </is>
-      </c>
-      <c r="C53" s="10" t="inlineStr">
-        <is>
-          <t>Manychat</t>
+          <t>Shopify</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>Maildoso</t>
+          <t>Klaviyo</t>
         </is>
       </c>
       <c r="G53" s="10" t="inlineStr">
         <is>
-          <t>Buffer</t>
+          <t>Social Media Analytics</t>
         </is>
       </c>
       <c r="H53" s="10" t="inlineStr">
         <is>
-          <t>Revenue Strategy</t>
+          <t>Pricing &amp; Packaging Strategy</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="B54" s="10" t="inlineStr">
-        <is>
-          <t>Shopify</t>
-        </is>
-      </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t>Klaviyo</t>
+          <t>Gohighlevel</t>
         </is>
       </c>
       <c r="G54" s="10" t="inlineStr">
         <is>
-          <t>Social Media Analytics</t>
-        </is>
-      </c>
-      <c r="H54" s="10" t="inlineStr">
-        <is>
-          <t>Pricing &amp; Packaging Strategy</t>
+          <t>Social Media Reporting</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t>Gohighlevel</t>
+          <t>Lemlist</t>
         </is>
       </c>
       <c r="G55" s="10" t="inlineStr">
         <is>
-          <t>Social Media Reporting</t>
+          <t>Social Media Dashboard</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t>Lemlist</t>
+          <t>Clay</t>
         </is>
       </c>
       <c r="G56" s="10" t="inlineStr">
         <is>
-          <t>Social Media Dashboard</t>
+          <t>Content Calendar</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="D57" s="10" t="inlineStr">
-        <is>
-          <t>Clay</t>
-        </is>
-      </c>
       <c r="G57" s="10" t="inlineStr">
         <is>
-          <t>Content Calendar</t>
+          <t>Social Media Automation</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="G58" s="10" t="inlineStr">
         <is>
-          <t>Social Media Automation</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="G59" s="10" t="inlineStr">
-        <is>
           <t>Google Analytics GA4</t>
         </is>
       </c>
     </row>
+    <row r="59"/>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>Genéricas (solo LinkedIn):</t>
+        </is>
+      </c>
+      <c r="B60" s="9" t="inlineStr">
+        <is>
+          <t>(SEARCH 1)</t>
+        </is>
+      </c>
+    </row>
     <row r="61">
-      <c r="A61" s="8" t="inlineStr">
-        <is>
-          <t>Genéricas (solo LinkedIn):</t>
-        </is>
-      </c>
-      <c r="B61" s="9" t="inlineStr">
-        <is>
-          <t>(SEARCH 1)</t>
+      <c r="B61" s="10" t="inlineStr">
+        <is>
+          <t>1099 contractor</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="B62" s="10" t="inlineStr">
-        <is>
-          <t>1099 contractor</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="B63" s="10" t="inlineStr">
         <is>
           <t>independent contractor</t>
         </is>

</xml_diff>

<commit_message>
doc(linkedin): Excel con 2 vistas de keywords (4 áreas del master + 8 Business Units)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/linkedin jobs/LinkedIn - Criterios y Keywords.xlsx
+++ b/linkedin jobs/LinkedIn - Criterios y Keywords.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Search Fields" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criterios" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Solapas y Estados" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por BU (8)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criterios" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Solapas y Estados" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,8 +62,13 @@
       <color rgb="001F1E1B"/>
       <sz val="10"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="006B6B65"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -95,6 +101,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006AA84F"/>
       </patternFill>
     </fill>
   </fills>
@@ -138,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -158,6 +169,8 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -543,7 +556,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -826,7 +838,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -1082,7 +1093,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
@@ -1359,7 +1369,6 @@
         </is>
       </c>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
@@ -1718,7 +1727,6 @@
         </is>
       </c>
     </row>
-    <row r="59"/>
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
@@ -1751,6 +1759,1448 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B206"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Keywords por Business Unit (Upwork + LinkedIn = mismas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>8 BU del classifier · LinkedIn suma filtro 1099 + US · 186 keywords</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Finance &amp; Accounting</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>45 keywords</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Financial Analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Head of Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Finance Director</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Financial Consultant</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Financial Advisor</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Financial Controller</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Financial Modeler</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Financial Models</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Forecast</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Cashflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Profit and Loss</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Financial Statement</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Profitability</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Balance Sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>Valuation</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Mergers and Acquisitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>IRR</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>MOIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>DCF</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>Business Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>Business Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Pitch Deck</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>Business Model</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>One pager</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>Financial Modelling</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>Financial Projection</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>Financial Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>Financial Planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>Financial Forecasting</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>Financial Planning and Budgeting</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>Financial Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>Fathom HQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>Floatapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>Baremetrics</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>Churnkey</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>Triple Whale</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>Income Statement</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>Scenario Planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>Sensitivity Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>Working Capital</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>Business Operations &amp; Back-Office</t>
+        </is>
+      </c>
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>35 keywords</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>Inventory Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="inlineStr">
+        <is>
+          <t>Warehouse Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>Demand Planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>Procurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="inlineStr">
+        <is>
+          <t>Vendor Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="10" t="inlineStr">
+        <is>
+          <t>Supply Chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="inlineStr">
+        <is>
+          <t>Xfin</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="10" t="inlineStr">
+        <is>
+          <t>Odoo</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="10" t="inlineStr">
+        <is>
+          <t>Xero</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="10" t="inlineStr">
+        <is>
+          <t>QuickBooks</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="10" t="inlineStr">
+        <is>
+          <t>Netsuite</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="10" t="inlineStr">
+        <is>
+          <t>ServiceTitan</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="10" t="inlineStr">
+        <is>
+          <t>Service Titan</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="10" t="inlineStr">
+        <is>
+          <t>QBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="10" t="inlineStr">
+        <is>
+          <t>Bank Reconciliation</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="10" t="inlineStr">
+        <is>
+          <t>Treasury Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="10" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="10" t="inlineStr">
+        <is>
+          <t>Corporate Advisory</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="10" t="inlineStr">
+        <is>
+          <t>Invoice Automation</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="10" t="inlineStr">
+        <is>
+          <t>Bookkeeper</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="10" t="inlineStr">
+        <is>
+          <t>Chart of Accounts</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="10" t="inlineStr">
+        <is>
+          <t>Books to Bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="10" t="inlineStr">
+        <is>
+          <t>Business Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="10" t="inlineStr">
+        <is>
+          <t>Business Development</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="10" t="inlineStr">
+        <is>
+          <t>Business Operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="10" t="inlineStr">
+        <is>
+          <t>Business Consulting</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="10" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="10" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="10" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="10" t="inlineStr">
+        <is>
+          <t>Pumping</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="10" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="10" t="inlineStr">
+        <is>
+          <t>Gyms</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="10" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="10" t="inlineStr">
+        <is>
+          <t>Laboratory</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="10" t="inlineStr">
+        <is>
+          <t>Clinic</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="11" t="inlineStr">
+        <is>
+          <t>Project Management &amp; BI</t>
+        </is>
+      </c>
+      <c r="B88" s="12" t="inlineStr">
+        <is>
+          <t>21 keywords</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="10" t="inlineStr">
+        <is>
+          <t>Project Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="10" t="inlineStr">
+        <is>
+          <t>Notion</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="10" t="inlineStr">
+        <is>
+          <t>Clickup</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="10" t="inlineStr">
+        <is>
+          <t>Asana</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="10" t="inlineStr">
+        <is>
+          <t>Jira</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="10" t="inlineStr">
+        <is>
+          <t>Reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="10" t="inlineStr">
+        <is>
+          <t>Business Intelligence</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="10" t="inlineStr">
+        <is>
+          <t>KPIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="10" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="10" t="inlineStr">
+        <is>
+          <t>Power BI</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="10" t="inlineStr">
+        <is>
+          <t>Looker Studio</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="10" t="inlineStr">
+        <is>
+          <t>Google Sheets</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="10" t="inlineStr">
+        <is>
+          <t>Big Query</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="10" t="inlineStr">
+        <is>
+          <t>Mysql</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="10" t="inlineStr">
+        <is>
+          <t>SQL</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="10" t="inlineStr">
+        <is>
+          <t>Pinecone</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="10" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="10" t="inlineStr">
+        <is>
+          <t>Snowflake</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="10" t="inlineStr">
+        <is>
+          <t>Data analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="10" t="inlineStr">
+        <is>
+          <t>Data Analytics</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="11" t="inlineStr">
+        <is>
+          <t>AI &amp; Automation</t>
+        </is>
+      </c>
+      <c r="B111" s="12" t="inlineStr">
+        <is>
+          <t>14 keywords</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="10" t="inlineStr">
+        <is>
+          <t>LLM</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="10" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="10" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="10" t="inlineStr">
+        <is>
+          <t>C++</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="10" t="inlineStr">
+        <is>
+          <t>NLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="10" t="inlineStr">
+        <is>
+          <t>Algorithms</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="10" t="inlineStr">
+        <is>
+          <t>Git</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="10" t="inlineStr">
+        <is>
+          <t>AI Agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="10" t="inlineStr">
+        <is>
+          <t>LangChain</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="10" t="inlineStr">
+        <is>
+          <t>LangGraph</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="10" t="inlineStr">
+        <is>
+          <t>AutoGen</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="10" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="10" t="inlineStr">
+        <is>
+          <t>Prompt Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="10" t="inlineStr">
+        <is>
+          <t>MCP</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="11" t="inlineStr">
+        <is>
+          <t>System Integrations</t>
+        </is>
+      </c>
+      <c r="B127" s="12" t="inlineStr">
+        <is>
+          <t>11 keywords</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="10" t="inlineStr">
+        <is>
+          <t>Automation</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="10" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="10" t="inlineStr">
+        <is>
+          <t>Scraping</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="10" t="inlineStr">
+        <is>
+          <t>Make.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="10" t="inlineStr">
+        <is>
+          <t>N8N</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="10" t="inlineStr">
+        <is>
+          <t>Zapier</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="10" t="inlineStr">
+        <is>
+          <t>Power Automate</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="10" t="inlineStr">
+        <is>
+          <t>Low Code</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="10" t="inlineStr">
+        <is>
+          <t>No Code</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="10" t="inlineStr">
+        <is>
+          <t>Airtable</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="10" t="inlineStr">
+        <is>
+          <t>Softr</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="11" t="inlineStr">
+        <is>
+          <t>Digital Experience &amp; Product Development</t>
+        </is>
+      </c>
+      <c r="B140" s="12" t="inlineStr">
+        <is>
+          <t>14 keywords</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="10" t="inlineStr">
+        <is>
+          <t>Web Development</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="10" t="inlineStr">
+        <is>
+          <t>Figma</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="10" t="inlineStr">
+        <is>
+          <t>Framer</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="10" t="inlineStr">
+        <is>
+          <t>Webflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="10" t="inlineStr">
+        <is>
+          <t>Wordpress</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="10" t="inlineStr">
+        <is>
+          <t>Woocommerce</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="10" t="inlineStr">
+        <is>
+          <t>E-commerce development</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="10" t="inlineStr">
+        <is>
+          <t>Shopify</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="10" t="inlineStr">
+        <is>
+          <t>Cursor</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="10" t="inlineStr">
+        <is>
+          <t>Lovable</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="10" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="10" t="inlineStr">
+        <is>
+          <t>App development</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="10" t="inlineStr">
+        <is>
+          <t>Bolt</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="11" t="inlineStr">
+        <is>
+          <t>Sales &amp; Customer Success</t>
+        </is>
+      </c>
+      <c r="B156" s="12" t="inlineStr">
+        <is>
+          <t>18 keywords</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="10" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="10" t="inlineStr">
+        <is>
+          <t>Hubspot</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="10" t="inlineStr">
+        <is>
+          <t>Zoho</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="10" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="10" t="inlineStr">
+        <is>
+          <t>Instantly</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="10" t="inlineStr">
+        <is>
+          <t>Manyreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="10" t="inlineStr">
+        <is>
+          <t>Manychat</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="10" t="inlineStr">
+        <is>
+          <t>Apollo</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="10" t="inlineStr">
+        <is>
+          <t>Email marketing</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="10" t="inlineStr">
+        <is>
+          <t>Lead Gen</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="10" t="inlineStr">
+        <is>
+          <t>Kommo</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="10" t="inlineStr">
+        <is>
+          <t>Bounceban</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="10" t="inlineStr">
+        <is>
+          <t>Twilio</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="10" t="inlineStr">
+        <is>
+          <t>Maildoso</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="10" t="inlineStr">
+        <is>
+          <t>Klaviyo</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="10" t="inlineStr">
+        <is>
+          <t>Gohighlevel</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="10" t="inlineStr">
+        <is>
+          <t>Lemlist</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="10" t="inlineStr">
+        <is>
+          <t>Clay</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="11" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Brand</t>
+        </is>
+      </c>
+      <c r="B176" s="12" t="inlineStr">
+        <is>
+          <t>26 keywords</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="10" t="inlineStr">
+        <is>
+          <t>Metricool</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="10" t="inlineStr">
+        <is>
+          <t>Supermetrics</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="10" t="inlineStr">
+        <is>
+          <t>Gamma</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="10" t="inlineStr">
+        <is>
+          <t>Canva</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="10" t="inlineStr">
+        <is>
+          <t>Liveplan</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="10" t="inlineStr">
+        <is>
+          <t>Campaign Outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="10" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="10" t="inlineStr">
+        <is>
+          <t>Linkedin Ads</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="10" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="10" t="inlineStr">
+        <is>
+          <t>Tiktok Ads</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="10" t="inlineStr">
+        <is>
+          <t>Hootsuite</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="10" t="inlineStr">
+        <is>
+          <t>Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="10" t="inlineStr">
+        <is>
+          <t>Social Media Analytics</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="10" t="inlineStr">
+        <is>
+          <t>Social Media Reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="10" t="inlineStr">
+        <is>
+          <t>Social Media Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="10" t="inlineStr">
+        <is>
+          <t>Content Calendar</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="10" t="inlineStr">
+        <is>
+          <t>Social Media Automation</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="10" t="inlineStr">
+        <is>
+          <t>Google Analytics GA4</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="10" t="inlineStr">
+        <is>
+          <t>Go-to-Market Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="10" t="inlineStr">
+        <is>
+          <t>GTM Framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="10" t="inlineStr">
+        <is>
+          <t>Market Entry Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="10" t="inlineStr">
+        <is>
+          <t>Product Launch Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="10" t="inlineStr">
+        <is>
+          <t>Growth Strategy Consultant</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="10" t="inlineStr">
+        <is>
+          <t>Commercial Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="10" t="inlineStr">
+        <is>
+          <t>Revenue Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="10" t="inlineStr">
+        <is>
+          <t>Pricing &amp; Packaging Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="11" t="inlineStr">
+        <is>
+          <t>Genéricas (todas las BU)</t>
+        </is>
+      </c>
+      <c r="B204" s="12" t="inlineStr">
+        <is>
+          <t>2 keywords</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="10" t="inlineStr">
+        <is>
+          <t>1099 contractor</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="10" t="inlineStr">
+        <is>
+          <t>independent contractor</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2037,7 +3487,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
doc(linkedin): solapa 'Upwork vs LinkedIn' (mismas keywords, distinto filtro)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/linkedin jobs/LinkedIn - Criterios y Keywords.xlsx
+++ b/linkedin jobs/LinkedIn - Criterios y Keywords.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por BU (8)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Search Fields" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criterios" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Solapas de la app" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upwork vs LinkedIn" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criterios" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Solapas de la app" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -57,7 +58,7 @@
       <color rgb="001F1E1B"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -99,6 +100,16 @@
         <fgColor rgb="00F1F2F4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000BA37F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002867B2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -126,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -164,6 +175,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -553,7 +570,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Genéricas (todas las BU): 1099 contractor · independent contractor · 186 keywords en total</t>
+          <t>Genéricas (todas las BU): 1099 contractor · independent contractor · 186 keywords en total  ·  MISMAS keywords en Upwork y LinkedIn</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1703,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mismas keywords que Upwork · LinkedIn suma filtro 1099 + US y rotación · 186 keywords</t>
+          <t>Mismas keywords que Upwork · LinkedIn suma filtro 1099 + US y rotación · 186 keywords  ·  MISMAS keywords en Upwork y LinkedIn</t>
         </is>
       </c>
     </row>
@@ -2867,6 +2884,227 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="000BA37F"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Upwork vs LinkedIn — mismo cerebro, distinto filtro</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Las keywords son IDÉNTICAS en las dos plataformas. Lo que cambia son los filtros y el volumen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Aspecto</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Upwork</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Keywords</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Las 186 (por Business Unit)</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Las MISMAS 186</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Cómo busca</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>API oficial de Upwork</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Guest API de LinkedIn (scraping)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>País</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>~20 países permitidos</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Solo Estados Unidos (fijo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Tipo de trabajo</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Cualquiera (con tarifa)</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>Contract/Freelance = 1099, excluye W2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Plata</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Piso /h</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>No da tarifa fija; se guarda el rango si viene</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Frescura</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Posteado ≤ 48h</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Última semana</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Volumen</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Alto (marketplace 100% freelance)</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Bajo (LinkedIn es mayormente full-time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>Corridas</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Cada 4h, 4 scrapers</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>Cada 4h, rotando 15 keywords</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Clasificación</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Classifier vs las 8 BU</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>El MISMO classifier vs las 8 BU</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>A dónde llega</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Check Proposal (si hace fit)</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>Check Proposal (si es 1099 US + fit)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00A64D79"/>
@@ -3110,7 +3348,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00674EA7"/>

</xml_diff>

<commit_message>
doc(linkedin): solapa Resumen para dirección (por qué por BU + 8 BU + mismas keywords Upwork/LinkedIn)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/linkedin jobs/LinkedIn - Criterios y Keywords.xlsx
+++ b/linkedin jobs/LinkedIn - Criterios y Keywords.xlsx
@@ -7,11 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por BU (8)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Search Fields" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upwork vs LinkedIn" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criterios" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Solapas de la app" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por BU (8)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Search Fields" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upwork vs LinkedIn" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criterios" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Solapas de la app" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +57,29 @@
     <font>
       <b val="1"/>
       <color rgb="001F1E1B"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F1E1B"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="004A4A45"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F1E1B"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="001F1E1B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="004A4A45"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="11">
@@ -137,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -180,6 +204,21 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -543,6 +582,165 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F1E1B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:B23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn CRM — Keywords por Business Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>Resumen para dirección</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>¿Por qué organizamos las keywords por Business Unit?</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44" customHeight="1">
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>Organizamos las keywords por las 8 Business Units (las mismas que usa el classifier) para que cada búsqueda quede alineada al servicio real de SWL que la va a captar, y no en bolsas genéricas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>Así se ve de un vistazo qué keywords alimentan cada BU, es fácil sumar o sacar términos por área, y queda un criterio único que sirve igual para Upwork y para LinkedIn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="44" customHeight="1">
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>Usamos las MISMAS keywords para Upwork y para LinkedIn; en LinkedIn sumamos el filtro obligatorio 1099 + US, y solo lo que hace fit con una BU llega a Check Proposal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>Las 8 Business Units:</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>1.  AI &amp; Automation</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>2.  Business Operations &amp; Back-Office</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>3.  Digital Experience &amp; Product Development</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>4.  Finance &amp; Accounting</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>5.  Marketing &amp; Brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>6.  Project Management &amp; BI</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>7.  Sales &amp; Customer Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="20" t="inlineStr">
+        <is>
+          <t>8.  System Integrations</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>En este archivo:</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="21" t="inlineStr">
+        <is>
+          <t>• Por BU (8): las 186 keywords repartidas en las 8 Business Units.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t>• Search Fields: las mismas keywords en el formato de áreas del master de Upwork.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="21" t="inlineStr">
+        <is>
+          <t>• Upwork vs LinkedIn: qué es igual y qué cambia entre las dos plataformas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>• Criterios / Solapas: reglas del pipeline y qué muestra cada vista de la app.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="0038761D"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -1673,7 +1871,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C27BA0"/>
@@ -2883,7 +3081,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="000BA37F"/>
@@ -3104,7 +3302,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00A64D79"/>
@@ -3348,7 +3546,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00674EA7"/>

</xml_diff>